<commit_message>
Correción de decimales en Invenrario
</commit_message>
<xml_diff>
--- a/Ejemplos/EJEMPLO_kardex_inventario.xlsx
+++ b/Ejemplos/EJEMPLO_kardex_inventario.xlsx
@@ -16,8 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="&quot;Bs&quot; #,##0.00"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="&quot;Bs&quot; #,##0.0"/>
+    <numFmt numFmtId="165" formatCode="&quot;Bs&quot; #,##0.00"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -72,7 +73,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -83,8 +84,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -554,19 +556,19 @@
       <c r="D5" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E5" s="5" t="n">
+      <c r="E5" s="6" t="n">
         <v>50</v>
       </c>
       <c r="F5" s="2" t="n"/>
       <c r="G5" s="5" t="n"/>
-      <c r="H5" s="5" t="n"/>
+      <c r="H5" s="6" t="n"/>
       <c r="I5" s="2" t="n">
         <v>10</v>
       </c>
       <c r="J5" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="K5" s="5" t="n">
+      <c r="K5" s="6" t="n">
         <v>50</v>
       </c>
     </row>
@@ -587,19 +589,19 @@
       <c r="D6" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="E6" s="5" t="n">
+      <c r="E6" s="6" t="n">
         <v>70</v>
       </c>
       <c r="F6" s="2" t="n"/>
       <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="n"/>
+      <c r="H6" s="6" t="n"/>
       <c r="I6" s="2" t="n">
         <v>20</v>
       </c>
       <c r="J6" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="K6" s="5" t="n">
+      <c r="K6" s="6" t="n">
         <v>120</v>
       </c>
     </row>
@@ -616,14 +618,14 @@
       </c>
       <c r="C7" s="2" t="n"/>
       <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5" t="n"/>
+      <c r="E7" s="6" t="n"/>
       <c r="F7" s="2" t="n">
         <v>5</v>
       </c>
       <c r="G7" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="H7" s="5" t="n">
+      <c r="H7" s="6" t="n">
         <v>30</v>
       </c>
       <c r="I7" s="2" t="n">
@@ -632,7 +634,7 @@
       <c r="J7" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="K7" s="5" t="n">
+      <c r="K7" s="6" t="n">
         <v>90</v>
       </c>
     </row>
@@ -653,38 +655,38 @@
       <c r="D8" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="E8" s="5" t="n">
+      <c r="E8" s="6" t="n">
         <v>40</v>
       </c>
       <c r="F8" s="2" t="n"/>
       <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="n"/>
+      <c r="H8" s="6" t="n"/>
       <c r="I8" s="2" t="n">
         <v>20</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>6.5</v>
       </c>
-      <c r="K8" s="5" t="n">
+      <c r="K8" s="6" t="n">
         <v>130</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C9" s="6" t="n">
+      <c r="C9" s="7" t="n">
         <v>25</v>
       </c>
-      <c r="E9" s="7" t="n">
+      <c r="E9" s="8" t="n">
         <v>160</v>
       </c>
-      <c r="F9" s="6" t="n">
+      <c r="F9" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="H9" s="7" t="n">
+      <c r="H9" s="8" t="n">
         <v>30</v>
       </c>
     </row>

</xml_diff>